<commit_message>
Day 08: FLOOR, CEILING, MROUND, ABS, MOD, POWER and SQRT
</commit_message>
<xml_diff>
--- a/Excel/Day 07/Excel-Practice-(Day-07).xlsx
+++ b/Excel/Day 07/Excel-Practice-(Day-07).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analyst\Excel\Day 07\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6FF0FB1-813A-4AFE-8248-7F2F0E0950BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCFEB30-F68B-4A62-ABA9-CC968EEF0874}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="11835" tabRatio="678" firstSheet="11" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="678" firstSheet="14" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -27,6 +27,8 @@
     <sheet name="Cell Referencing" sheetId="13" r:id="rId12"/>
     <sheet name="Text Formulas Notes" sheetId="14" r:id="rId13"/>
     <sheet name="Text Formulas Practice" sheetId="15" r:id="rId14"/>
+    <sheet name="Statistical Formulas Notes" sheetId="16" r:id="rId15"/>
+    <sheet name="Statistical Formulas Practice" sheetId="17" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Filter!$A$1:$F$38</definedName>
@@ -41,8 +43,8 @@
     </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{46BE6895-7355-4a93-B00E-2C351335B9C9}">
       <x15:slicerCaches xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main">
-        <x14:slicerCache r:id="rId15"/>
-        <x14:slicerCache r:id="rId16"/>
+        <x14:slicerCache r:id="rId17"/>
+        <x14:slicerCache r:id="rId18"/>
       </x15:slicerCaches>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -62,7 +64,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -84,7 +86,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4203" uniqueCount="752">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4385" uniqueCount="907">
   <si>
     <t>Employee_ID</t>
   </si>
@@ -2341,6 +2343,471 @@
   </si>
   <si>
     <t>%$</t>
+  </si>
+  <si>
+    <t>Meaning</t>
+  </si>
+  <si>
+    <t>AVERAGE</t>
+  </si>
+  <si>
+    <t>AVERAGE(range)</t>
+  </si>
+  <si>
+    <t>Average nikaalta hai</t>
+  </si>
+  <si>
+    <t>Mean calculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =AVERAGE(10,20,30) → 20</t>
+  </si>
+  <si>
+    <t>MAX</t>
+  </si>
+  <si>
+    <t>MAX(range)</t>
+  </si>
+  <si>
+    <t>Sabse badi value</t>
+  </si>
+  <si>
+    <t>Highest find</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =MAX(10,50,30) → 50</t>
+  </si>
+  <si>
+    <t>MIN</t>
+  </si>
+  <si>
+    <t>MIN(range)</t>
+  </si>
+  <si>
+    <t>Sabse chhoti value</t>
+  </si>
+  <si>
+    <t>Lowest find</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =MIN(10,50,30) → 10</t>
+  </si>
+  <si>
+    <t>COUNT</t>
+  </si>
+  <si>
+    <t>COUNT(range)</t>
+  </si>
+  <si>
+    <t>Numeric cells count karta hai</t>
+  </si>
+  <si>
+    <t>Numbers count</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =COUNT(1,2,"A") → 2</t>
+  </si>
+  <si>
+    <t>COUNTA</t>
+  </si>
+  <si>
+    <t>COUNTA(range)</t>
+  </si>
+  <si>
+    <t>Non-empty cells count karta hai</t>
+  </si>
+  <si>
+    <t>Filled cells</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =COUNTA(1,"A") → 2</t>
+  </si>
+  <si>
+    <t>COUNTIF</t>
+  </si>
+  <si>
+    <t>COUNTIF(range, criteria)</t>
+  </si>
+  <si>
+    <t>Condition par count karta hai</t>
+  </si>
+  <si>
+    <t>Conditional count</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =COUNTIF(A1,"&gt;50")</t>
+  </si>
+  <si>
+    <t>COUNTIFS</t>
+  </si>
+  <si>
+    <t>COUNTIFS(range1, criteria1, ...)</t>
+  </si>
+  <si>
+    <t>Multiple conditions par count karta hai</t>
+  </si>
+  <si>
+    <t>Advanced filtering</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =COUNTIFS(A1,"&gt;50",B1,"Pass")</t>
+  </si>
+  <si>
+    <t>AVERAGEIF</t>
+  </si>
+  <si>
+    <t>AVERAGEIF(range, criteria)</t>
+  </si>
+  <si>
+    <t>Condition par average karta hai</t>
+  </si>
+  <si>
+    <t>Filtered average</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =AVERAGEIF(A1,"&gt;50")</t>
+  </si>
+  <si>
+    <t>AVERAGEIFS</t>
+  </si>
+  <si>
+    <t>AVERAGEIFS(avg_range, criteria_range1, criteria1, ...)</t>
+  </si>
+  <si>
+    <t>Multiple conditions par average karta hai</t>
+  </si>
+  <si>
+    <t>Advanced average</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =AVERAGEIFS(C1,A1,"&gt;50")</t>
+  </si>
+  <si>
+    <t>SUM</t>
+  </si>
+  <si>
+    <t>SUM(range)</t>
+  </si>
+  <si>
+    <t>Total sum karta hai</t>
+  </si>
+  <si>
+    <t>Total calculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =SUM(10,20,30) → 60</t>
+  </si>
+  <si>
+    <t>SUMIF</t>
+  </si>
+  <si>
+    <t>SUMIF(range, criteria, sum_range)</t>
+  </si>
+  <si>
+    <t>Condition par sum karta hai</t>
+  </si>
+  <si>
+    <t>Conditional total</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =SUMIF(A1,"&gt;50",B1)</t>
+  </si>
+  <si>
+    <t>SUMIFS</t>
+  </si>
+  <si>
+    <t>SUMIFS(sum_range, criteria_range1, criteria1, ...)</t>
+  </si>
+  <si>
+    <t>Multiple conditions par sum karta hai</t>
+  </si>
+  <si>
+    <t>Complex analysis</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =SUMIFS(C1,A1,"&gt;50",B1,"Pass")</t>
+  </si>
+  <si>
+    <t>LARGE</t>
+  </si>
+  <si>
+    <t>LARGE(range, k)</t>
+  </si>
+  <si>
+    <t>K-th largest value</t>
+  </si>
+  <si>
+    <t>Top values</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =LARGE(A1,2)</t>
+  </si>
+  <si>
+    <t>SMALL</t>
+  </si>
+  <si>
+    <t>SMALL(range, k)</t>
+  </si>
+  <si>
+    <t>K-th smallest value</t>
+  </si>
+  <si>
+    <t>Bottom values</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =SMALL(A1,2)</t>
+  </si>
+  <si>
+    <t>RANK</t>
+  </si>
+  <si>
+    <t>RANK(number, range)</t>
+  </si>
+  <si>
+    <t>Rank deta hai</t>
+  </si>
+  <si>
+    <t>Position</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =RANK(80,A1)</t>
+  </si>
+  <si>
+    <t>ROUND</t>
+  </si>
+  <si>
+    <t>ROUND(number, num_digits)</t>
+  </si>
+  <si>
+    <t>Normal rounding</t>
+  </si>
+  <si>
+    <t>Approximate value</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =ROUND(12.345,2) → 12.35</t>
+  </si>
+  <si>
+    <t>ROUNDUP</t>
+  </si>
+  <si>
+    <t>ROUNDUP(number, num_digits)</t>
+  </si>
+  <si>
+    <t>Zero se door round karta hai</t>
+  </si>
+  <si>
+    <t>Always round away from zero</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =ROUNDUP(12.341,2) → 12.35</t>
+  </si>
+  <si>
+    <t>ROUNDDOWN</t>
+  </si>
+  <si>
+    <t>ROUNDDOWN(number, num_digits)</t>
+  </si>
+  <si>
+    <t>Zero ki taraf round karta hai</t>
+  </si>
+  <si>
+    <t>Rounding down</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =ROUNDDOWN(12.349,2) → 12.34</t>
+  </si>
+  <si>
+    <t>INT</t>
+  </si>
+  <si>
+    <t>INT(number)</t>
+  </si>
+  <si>
+    <t>Lower integer deta hai</t>
+  </si>
+  <si>
+    <t>Integer conversion</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =INT(12.9) → 12</t>
+  </si>
+  <si>
+    <t>TRUNC</t>
+  </si>
+  <si>
+    <t>TRUNC(number, [digits])</t>
+  </si>
+  <si>
+    <t>Decimal digits cut karta hai</t>
+  </si>
+  <si>
+    <t>Exact truncation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =TRUNC(12.987,2) → 12.98</t>
+  </si>
+  <si>
+    <t>FLOOR</t>
+  </si>
+  <si>
+    <t>FLOOR(number, significance)</t>
+  </si>
+  <si>
+    <t>Lower multiple tak round karta hai</t>
+  </si>
+  <si>
+    <t>Lower multiple</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =FLOOR(23,5) → 20</t>
+  </si>
+  <si>
+    <t>MROUND</t>
+  </si>
+  <si>
+    <t>MROUND(number, multiple)</t>
+  </si>
+  <si>
+    <t>Nearest multiple tak round karta hai</t>
+  </si>
+  <si>
+    <t>Smart rounding</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =MROUND(23,5) → 25</t>
+  </si>
+  <si>
+    <t>RAND</t>
+  </si>
+  <si>
+    <t>RAND()</t>
+  </si>
+  <si>
+    <t>Random decimal deta hai</t>
+  </si>
+  <si>
+    <t>Random data</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =RAND()</t>
+  </si>
+  <si>
+    <t>RANDBETWEEN</t>
+  </si>
+  <si>
+    <t>RANDBETWEEN(bottom, top)</t>
+  </si>
+  <si>
+    <t>Random integer deta hai</t>
+  </si>
+  <si>
+    <t>Testing data</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =RANDBETWEEN(1,100)</t>
+  </si>
+  <si>
+    <t>RANDARRAY</t>
+  </si>
+  <si>
+    <t>RANDARRAY(rows, cols, min, max, integer)</t>
+  </si>
+  <si>
+    <t>Random numbers ki table banata hai</t>
+  </si>
+  <si>
+    <t>Bulk data</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =RANDARRAY(5,3,1,100,TRUE)</t>
+  </si>
+  <si>
+    <t>ABS</t>
+  </si>
+  <si>
+    <t>ABS(number)</t>
+  </si>
+  <si>
+    <t>Absolute value deta hai</t>
+  </si>
+  <si>
+    <t>Distance calculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =ABS(-10) → 10</t>
+  </si>
+  <si>
+    <t>MOD</t>
+  </si>
+  <si>
+    <t>MOD(number, divisor)</t>
+  </si>
+  <si>
+    <t>Remainder deta hai</t>
+  </si>
+  <si>
+    <t>Even/odd check</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =MOD(10,3) → 1</t>
+  </si>
+  <si>
+    <t>POWER</t>
+  </si>
+  <si>
+    <t>POWER(number, power)</t>
+  </si>
+  <si>
+    <t>Power nikaalta hai</t>
+  </si>
+  <si>
+    <t>Exponential calculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =POWER(2,3) → 8</t>
+  </si>
+  <si>
+    <t>SQRT</t>
+  </si>
+  <si>
+    <t>SQRT(number)</t>
+  </si>
+  <si>
+    <t>Square root nikaalta hai</t>
+  </si>
+  <si>
+    <t>Math calculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> =SQRT(16) → 4</t>
+  </si>
+  <si>
+    <t>Statistical, rounding, random and mathematical formulas reference</t>
+  </si>
+  <si>
+    <t>Rand (0 to 1)</t>
+  </si>
+  <si>
+    <t>RANDBETWEEN(TOP,BOTTOM)</t>
+  </si>
+  <si>
+    <t>S.NO</t>
+  </si>
+  <si>
+    <t>NUMBERS</t>
+  </si>
+  <si>
+    <t>ROUND UP</t>
+  </si>
+  <si>
+    <t>ROUND DOWN</t>
+  </si>
+  <si>
+    <t>INTEGER</t>
+  </si>
+  <si>
+    <t>INTEGER,TRUNC</t>
   </si>
 </sst>
 </file>
@@ -2354,7 +2821,7 @@
     <numFmt numFmtId="167" formatCode="&quot;Rs. &quot;#,##0"/>
     <numFmt numFmtId="168" formatCode="&quot;Rs.&quot;\ #,##0"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2551,8 +3018,28 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="31">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2732,8 +3219,32 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA9D3E5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4B183"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF70AD47"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="54">
+  <borders count="70">
     <border>
       <left/>
       <right/>
@@ -3426,12 +3937,182 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF1F1F1F"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF1F1F1F"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF1F1F1F"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF1F1F1F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1F1F1F"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1F1F1F"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF548235"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF548235"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF808080"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF548235"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF548235"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF548235"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="211">
+  <cellXfs count="265">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3983,12 +4664,324 @@
     <xf numFmtId="0" fontId="21" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="57" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="60" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="61" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="63" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="61" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="61" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="62" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="31" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="62" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="32" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="64" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="68" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="61" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="67" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="61" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="62" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="63" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="61" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="66" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="61" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="62" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="63" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="58">
+  <dxfs count="73">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5870,15 +6863,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}" name="Employees" displayName="Employees" ref="A1:F39" totalsRowCount="1" headerRowDxfId="43" dataDxfId="41" headerRowBorderDxfId="42" tableBorderDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}" name="Employees" displayName="Employees" ref="A1:F39" totalsRowCount="1" headerRowDxfId="58" dataDxfId="56" headerRowBorderDxfId="57" tableBorderDxfId="55">
   <autoFilter ref="A1:F38" xr:uid="{2688C5AF-1E0A-4EDD-AF11-5A4BBABB9721}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{B1033A5F-C26D-48E8-B4BE-5F7761A770FB}" name="Date" dataDxfId="39" totalsRowDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{AD6BA12D-25CE-4D3E-8E2A-1DD281A3FDA5}" name="Employee Name" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="3" xr3:uid="{96E1CF2B-482C-42D2-8CEA-C0CE6D69979C}" name="Department" dataDxfId="35" totalsRowDxfId="34"/>
-    <tableColumn id="4" xr3:uid="{602E6D48-4D10-4D1E-9636-6A41FF0A4753}" name="Region" dataDxfId="33" totalsRowDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{98D904BD-DEE8-4674-A97B-995E27B5AB23}" name="Sales (Rs.)" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="6" xr3:uid="{F7A5EC06-42D8-4DD0-83BA-C91339988D38}" name="Target (Rs.)" totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="28">
+    <tableColumn id="1" xr3:uid="{B1033A5F-C26D-48E8-B4BE-5F7761A770FB}" name="Date" dataDxfId="54" totalsRowDxfId="53"/>
+    <tableColumn id="2" xr3:uid="{AD6BA12D-25CE-4D3E-8E2A-1DD281A3FDA5}" name="Employee Name" dataDxfId="52" totalsRowDxfId="51"/>
+    <tableColumn id="3" xr3:uid="{96E1CF2B-482C-42D2-8CEA-C0CE6D69979C}" name="Department" dataDxfId="50" totalsRowDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{602E6D48-4D10-4D1E-9636-6A41FF0A4753}" name="Region" dataDxfId="48" totalsRowDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{98D904BD-DEE8-4674-A97B-995E27B5AB23}" name="Sales (Rs.)" dataDxfId="46" totalsRowDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{F7A5EC06-42D8-4DD0-83BA-C91339988D38}" name="Target (Rs.)" totalsRowFunction="custom" dataDxfId="44" totalsRowDxfId="43">
       <totalsRowFormula>SUM(F2:F38)</totalsRowFormula>
     </tableColumn>
   </tableColumns>
@@ -6171,7 +7164,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="2">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -18673,7 +19666,7 @@
       </c>
       <c r="H3" s="135">
         <f t="shared" ref="H3:H16" ca="1" si="1">(RANDBETWEEN(10,50))/100</f>
-        <v>0.38</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="I3" s="105">
         <v>100</v>
@@ -18718,7 +19711,7 @@
       </c>
       <c r="H4" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.33</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="X4" s="105" t="str">
         <f t="shared" si="0"/>
@@ -18738,7 +19731,7 @@
       </c>
       <c r="AB4" s="135">
         <f t="shared" ca="1" si="2"/>
-        <v>0.38</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="AC4" s="105">
         <f t="shared" si="2"/>
@@ -18760,7 +19753,7 @@
       </c>
       <c r="H5" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.17</v>
+        <v>0.43</v>
       </c>
       <c r="X5" s="105" t="str">
         <f t="shared" si="0"/>
@@ -18780,7 +19773,7 @@
       </c>
       <c r="AB5" s="135">
         <f t="shared" ref="AB5:AB17" ca="1" si="6">H4</f>
-        <v>0.33</v>
+        <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="6" spans="4:29" x14ac:dyDescent="0.25">
@@ -18798,7 +19791,7 @@
       </c>
       <c r="H6" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.11</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="L6" s="196" t="s">
         <v>540</v>
@@ -18830,7 +19823,7 @@
       </c>
       <c r="AB6" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.17</v>
+        <v>0.43</v>
       </c>
     </row>
     <row r="7" spans="4:29" x14ac:dyDescent="0.25">
@@ -18848,7 +19841,7 @@
       </c>
       <c r="H7" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.28999999999999998</v>
+        <v>0.13</v>
       </c>
       <c r="X7" s="105" t="str">
         <f t="shared" si="0"/>
@@ -18868,7 +19861,7 @@
       </c>
       <c r="AB7" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.11</v>
+        <v>0.28999999999999998</v>
       </c>
     </row>
     <row r="8" spans="4:29" x14ac:dyDescent="0.25">
@@ -18886,7 +19879,7 @@
       </c>
       <c r="H8" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.34</v>
+        <v>0.25</v>
       </c>
       <c r="M8" s="105">
         <v>137196</v>
@@ -18912,7 +19905,7 @@
       </c>
       <c r="AB8" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.28999999999999998</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="9" spans="4:29" x14ac:dyDescent="0.25">
@@ -18930,7 +19923,7 @@
       </c>
       <c r="H9" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.49</v>
+        <v>0.2</v>
       </c>
       <c r="M9" s="105">
         <v>64256</v>
@@ -18954,7 +19947,7 @@
       </c>
       <c r="AB9" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.34</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="10" spans="4:29" x14ac:dyDescent="0.25">
@@ -18972,7 +19965,7 @@
       </c>
       <c r="H10" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.27</v>
+        <v>0.19</v>
       </c>
       <c r="M10" s="105">
         <v>137080</v>
@@ -18998,7 +19991,7 @@
       </c>
       <c r="AB10" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.49</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="11" spans="4:29" x14ac:dyDescent="0.25">
@@ -19016,7 +20009,7 @@
       </c>
       <c r="H11" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.5</v>
+        <v>0.16</v>
       </c>
       <c r="M11" s="105">
         <v>95302</v>
@@ -19042,7 +20035,7 @@
       </c>
       <c r="AB11" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.27</v>
+        <v>0.19</v>
       </c>
     </row>
     <row r="12" spans="4:29" x14ac:dyDescent="0.25">
@@ -19086,7 +20079,7 @@
       </c>
       <c r="AB12" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.5</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="13" spans="4:29" x14ac:dyDescent="0.25">
@@ -19104,7 +20097,7 @@
       </c>
       <c r="H13" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.24</v>
+        <v>0.11</v>
       </c>
       <c r="M13" s="105">
         <v>66062</v>
@@ -19148,7 +20141,7 @@
       </c>
       <c r="H14" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.32</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="M14" s="105">
         <v>98878</v>
@@ -19174,7 +20167,7 @@
       </c>
       <c r="AB14" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.24</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="15" spans="4:29" x14ac:dyDescent="0.25">
@@ -19192,7 +20185,7 @@
       </c>
       <c r="H15" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.34</v>
+        <v>0.31</v>
       </c>
       <c r="M15" s="105">
         <v>40851</v>
@@ -19218,7 +20211,7 @@
       </c>
       <c r="AB15" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.32</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="16" spans="4:29" x14ac:dyDescent="0.25">
@@ -19236,7 +20229,7 @@
       </c>
       <c r="H16" s="135">
         <f t="shared" ca="1" si="1"/>
-        <v>0.49</v>
+        <v>0.17</v>
       </c>
       <c r="M16" s="105"/>
       <c r="N16" s="105"/>
@@ -19258,7 +20251,7 @@
       </c>
       <c r="AB16" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.34</v>
+        <v>0.31</v>
       </c>
     </row>
     <row r="17" spans="4:28" x14ac:dyDescent="0.25">
@@ -19287,7 +20280,7 @@
       </c>
       <c r="AB17" s="135">
         <f t="shared" ca="1" si="6"/>
-        <v>0.49</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="18" spans="4:28" x14ac:dyDescent="0.25">
@@ -22278,104 +23271,104 @@
     <mergeCell ref="W4:AB4"/>
   </mergeCells>
   <conditionalFormatting sqref="E7:E56">
-    <cfRule type="cellIs" dxfId="27" priority="37" operator="equal">
+    <cfRule type="cellIs" dxfId="42" priority="37" operator="equal">
       <formula>20000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="38" operator="between">
+    <cfRule type="cellIs" dxfId="41" priority="38" operator="between">
       <formula>50000</formula>
       <formula>100000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="39" operator="between">
+    <cfRule type="cellIs" dxfId="40" priority="39" operator="between">
       <formula>"Rs. 65,984"</formula>
       <formula>"Rs. 121,395"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="40" operator="lessThan">
+    <cfRule type="cellIs" dxfId="39" priority="40" operator="lessThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="23" priority="41" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="41" operator="greaterThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="42" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="37" priority="42" operator="greaterThan">
       <formula>"Rs. 93,689"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:B56">
-    <cfRule type="containsText" dxfId="21" priority="36" operator="containsText" text="Ayesha khan">
+    <cfRule type="containsText" dxfId="36" priority="36" operator="containsText" text="Ayesha khan">
       <formula>NOT(ISERROR(SEARCH("Ayesha khan",B7)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A8:A56">
-    <cfRule type="timePeriod" dxfId="20" priority="34" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="35" priority="34" timePeriod="yesterday">
       <formula>FLOOR(A8,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="19" priority="35" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="34" priority="35" timePeriod="yesterday">
       <formula>FLOOR(A8,1)=TODAY()-1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A7:A56">
-    <cfRule type="timePeriod" dxfId="18" priority="31" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="33" priority="31" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A7,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A7,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="17" priority="32" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="32" priority="32" timePeriod="yesterday">
       <formula>FLOOR(A7,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="16" priority="33" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="31" priority="33" timePeriod="today">
       <formula>FLOOR(A7,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F7:F56">
-    <cfRule type="uniqueValues" dxfId="15" priority="29"/>
-    <cfRule type="duplicateValues" dxfId="14" priority="30"/>
+    <cfRule type="uniqueValues" dxfId="30" priority="29"/>
+    <cfRule type="duplicateValues" dxfId="29" priority="30"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="T7:T56">
-    <cfRule type="cellIs" dxfId="13" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="9" operator="equal">
       <formula>20000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="10" operator="between">
+    <cfRule type="cellIs" dxfId="27" priority="10" operator="between">
       <formula>50000</formula>
       <formula>100000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="11" priority="11" operator="between">
+    <cfRule type="cellIs" dxfId="26" priority="11" operator="between">
       <formula>"Rs. 65,984"</formula>
       <formula>"Rs. 121,395"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="12" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="12" operator="lessThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="13" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="13" operator="greaterThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="14" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="14" operator="greaterThan">
       <formula>"Rs. 93,689"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q7:Q56">
-    <cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="Ayesha khan">
+    <cfRule type="containsText" dxfId="22" priority="8" operator="containsText" text="Ayesha khan">
       <formula>NOT(ISERROR(SEARCH("Ayesha khan",Q7)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P8:P56">
-    <cfRule type="timePeriod" dxfId="6" priority="6" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="21" priority="6" timePeriod="yesterday">
       <formula>FLOOR(P8,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="5" priority="7" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="20" priority="7" timePeriod="yesterday">
       <formula>FLOOR(P8,1)=TODAY()-1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P7:P56">
-    <cfRule type="timePeriod" dxfId="4" priority="3" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="19" priority="3" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(P7,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(P7,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="3" priority="4" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="18" priority="4" timePeriod="yesterday">
       <formula>FLOOR(P7,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="2" priority="5" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="17" priority="5" timePeriod="today">
       <formula>FLOOR(P7,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U7:U56">
-    <cfRule type="uniqueValues" dxfId="1" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="uniqueValues" dxfId="16" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -26078,6 +27071,1864 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B54A3611-4A04-4C13-950D-B1A57B926186}">
+  <dimension ref="B3:G33"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" customWidth="1"/>
+    <col min="3" max="3" width="18.140625" customWidth="1"/>
+    <col min="4" max="5" width="36.140625" customWidth="1"/>
+    <col min="6" max="6" width="28.5703125" customWidth="1"/>
+    <col min="7" max="7" width="41.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" s="213" t="s">
+        <v>559</v>
+      </c>
+      <c r="C3" s="211" t="s">
+        <v>560</v>
+      </c>
+      <c r="D3" s="211" t="s">
+        <v>561</v>
+      </c>
+      <c r="E3" s="211" t="s">
+        <v>752</v>
+      </c>
+      <c r="F3" s="211" t="s">
+        <v>562</v>
+      </c>
+      <c r="G3" s="214" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" s="226">
+        <v>1</v>
+      </c>
+      <c r="C4" s="224" t="s">
+        <v>753</v>
+      </c>
+      <c r="D4" s="215" t="s">
+        <v>754</v>
+      </c>
+      <c r="E4" s="215" t="s">
+        <v>755</v>
+      </c>
+      <c r="F4" s="215" t="s">
+        <v>756</v>
+      </c>
+      <c r="G4" s="216" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" s="227">
+        <v>2</v>
+      </c>
+      <c r="C5" s="225" t="s">
+        <v>758</v>
+      </c>
+      <c r="D5" s="212" t="s">
+        <v>759</v>
+      </c>
+      <c r="E5" s="212" t="s">
+        <v>760</v>
+      </c>
+      <c r="F5" s="212" t="s">
+        <v>761</v>
+      </c>
+      <c r="G5" s="217" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B6" s="227">
+        <v>3</v>
+      </c>
+      <c r="C6" s="225" t="s">
+        <v>763</v>
+      </c>
+      <c r="D6" s="212" t="s">
+        <v>764</v>
+      </c>
+      <c r="E6" s="212" t="s">
+        <v>765</v>
+      </c>
+      <c r="F6" s="212" t="s">
+        <v>766</v>
+      </c>
+      <c r="G6" s="217" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="227">
+        <v>4</v>
+      </c>
+      <c r="C7" s="225" t="s">
+        <v>768</v>
+      </c>
+      <c r="D7" s="212" t="s">
+        <v>769</v>
+      </c>
+      <c r="E7" s="212" t="s">
+        <v>770</v>
+      </c>
+      <c r="F7" s="212" t="s">
+        <v>771</v>
+      </c>
+      <c r="G7" s="217" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="227">
+        <v>5</v>
+      </c>
+      <c r="C8" s="225" t="s">
+        <v>773</v>
+      </c>
+      <c r="D8" s="212" t="s">
+        <v>774</v>
+      </c>
+      <c r="E8" s="212" t="s">
+        <v>775</v>
+      </c>
+      <c r="F8" s="212" t="s">
+        <v>776</v>
+      </c>
+      <c r="G8" s="217" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B9" s="227">
+        <v>6</v>
+      </c>
+      <c r="C9" s="225" t="s">
+        <v>778</v>
+      </c>
+      <c r="D9" s="212" t="s">
+        <v>779</v>
+      </c>
+      <c r="E9" s="212" t="s">
+        <v>780</v>
+      </c>
+      <c r="F9" s="212" t="s">
+        <v>781</v>
+      </c>
+      <c r="G9" s="217" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B10" s="227">
+        <v>7</v>
+      </c>
+      <c r="C10" s="225" t="s">
+        <v>783</v>
+      </c>
+      <c r="D10" s="212" t="s">
+        <v>784</v>
+      </c>
+      <c r="E10" s="212" t="s">
+        <v>785</v>
+      </c>
+      <c r="F10" s="212" t="s">
+        <v>786</v>
+      </c>
+      <c r="G10" s="217" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="227">
+        <v>8</v>
+      </c>
+      <c r="C11" s="225" t="s">
+        <v>788</v>
+      </c>
+      <c r="D11" s="212" t="s">
+        <v>789</v>
+      </c>
+      <c r="E11" s="212" t="s">
+        <v>790</v>
+      </c>
+      <c r="F11" s="212" t="s">
+        <v>791</v>
+      </c>
+      <c r="G11" s="217" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="227">
+        <v>9</v>
+      </c>
+      <c r="C12" s="225" t="s">
+        <v>793</v>
+      </c>
+      <c r="D12" s="212" t="s">
+        <v>794</v>
+      </c>
+      <c r="E12" s="212" t="s">
+        <v>795</v>
+      </c>
+      <c r="F12" s="212" t="s">
+        <v>796</v>
+      </c>
+      <c r="G12" s="217" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B13" s="230">
+        <v>10</v>
+      </c>
+      <c r="C13" s="231" t="s">
+        <v>798</v>
+      </c>
+      <c r="D13" s="218" t="s">
+        <v>799</v>
+      </c>
+      <c r="E13" s="218" t="s">
+        <v>800</v>
+      </c>
+      <c r="F13" s="218" t="s">
+        <v>801</v>
+      </c>
+      <c r="G13" s="220" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B14" s="229">
+        <v>11</v>
+      </c>
+      <c r="C14" s="228" t="s">
+        <v>803</v>
+      </c>
+      <c r="D14" s="219" t="s">
+        <v>804</v>
+      </c>
+      <c r="E14" s="219" t="s">
+        <v>805</v>
+      </c>
+      <c r="F14" s="219" t="s">
+        <v>806</v>
+      </c>
+      <c r="G14" s="221" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B15" s="229">
+        <v>12</v>
+      </c>
+      <c r="C15" s="228" t="s">
+        <v>808</v>
+      </c>
+      <c r="D15" s="219" t="s">
+        <v>809</v>
+      </c>
+      <c r="E15" s="219" t="s">
+        <v>810</v>
+      </c>
+      <c r="F15" s="219" t="s">
+        <v>811</v>
+      </c>
+      <c r="G15" s="221" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B16" s="245">
+        <v>13</v>
+      </c>
+      <c r="C16" s="246" t="s">
+        <v>813</v>
+      </c>
+      <c r="D16" s="247" t="s">
+        <v>814</v>
+      </c>
+      <c r="E16" s="247" t="s">
+        <v>815</v>
+      </c>
+      <c r="F16" s="247" t="s">
+        <v>816</v>
+      </c>
+      <c r="G16" s="248" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B17" s="245">
+        <v>14</v>
+      </c>
+      <c r="C17" s="246" t="s">
+        <v>818</v>
+      </c>
+      <c r="D17" s="247" t="s">
+        <v>819</v>
+      </c>
+      <c r="E17" s="247" t="s">
+        <v>820</v>
+      </c>
+      <c r="F17" s="247" t="s">
+        <v>821</v>
+      </c>
+      <c r="G17" s="248" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B18" s="229">
+        <v>15</v>
+      </c>
+      <c r="C18" s="228" t="s">
+        <v>823</v>
+      </c>
+      <c r="D18" s="219" t="s">
+        <v>824</v>
+      </c>
+      <c r="E18" s="219" t="s">
+        <v>825</v>
+      </c>
+      <c r="F18" s="219" t="s">
+        <v>826</v>
+      </c>
+      <c r="G18" s="221" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B19" s="257">
+        <v>16</v>
+      </c>
+      <c r="C19" s="258" t="s">
+        <v>828</v>
+      </c>
+      <c r="D19" s="259" t="s">
+        <v>829</v>
+      </c>
+      <c r="E19" s="259" t="s">
+        <v>830</v>
+      </c>
+      <c r="F19" s="259" t="s">
+        <v>831</v>
+      </c>
+      <c r="G19" s="260" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B20" s="261">
+        <v>17</v>
+      </c>
+      <c r="C20" s="262" t="s">
+        <v>833</v>
+      </c>
+      <c r="D20" s="263" t="s">
+        <v>834</v>
+      </c>
+      <c r="E20" s="263" t="s">
+        <v>835</v>
+      </c>
+      <c r="F20" s="263" t="s">
+        <v>836</v>
+      </c>
+      <c r="G20" s="264" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B21" s="257">
+        <v>18</v>
+      </c>
+      <c r="C21" s="258" t="s">
+        <v>838</v>
+      </c>
+      <c r="D21" s="259" t="s">
+        <v>839</v>
+      </c>
+      <c r="E21" s="259" t="s">
+        <v>840</v>
+      </c>
+      <c r="F21" s="259" t="s">
+        <v>841</v>
+      </c>
+      <c r="G21" s="260" t="s">
+        <v>842</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B22" s="233">
+        <v>19</v>
+      </c>
+      <c r="C22" s="232" t="s">
+        <v>843</v>
+      </c>
+      <c r="D22" s="222" t="s">
+        <v>844</v>
+      </c>
+      <c r="E22" s="222" t="s">
+        <v>845</v>
+      </c>
+      <c r="F22" s="222" t="s">
+        <v>846</v>
+      </c>
+      <c r="G22" s="223" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B23" s="233">
+        <v>20</v>
+      </c>
+      <c r="C23" s="232" t="s">
+        <v>848</v>
+      </c>
+      <c r="D23" s="222" t="s">
+        <v>849</v>
+      </c>
+      <c r="E23" s="222" t="s">
+        <v>850</v>
+      </c>
+      <c r="F23" s="222" t="s">
+        <v>851</v>
+      </c>
+      <c r="G23" s="223" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B24" s="233">
+        <v>21</v>
+      </c>
+      <c r="C24" s="232" t="s">
+        <v>853</v>
+      </c>
+      <c r="D24" s="222" t="s">
+        <v>854</v>
+      </c>
+      <c r="E24" s="222" t="s">
+        <v>855</v>
+      </c>
+      <c r="F24" s="222" t="s">
+        <v>856</v>
+      </c>
+      <c r="G24" s="223" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B25" s="233">
+        <v>22</v>
+      </c>
+      <c r="C25" s="232" t="s">
+        <v>858</v>
+      </c>
+      <c r="D25" s="222" t="s">
+        <v>859</v>
+      </c>
+      <c r="E25" s="222" t="s">
+        <v>860</v>
+      </c>
+      <c r="F25" s="222" t="s">
+        <v>861</v>
+      </c>
+      <c r="G25" s="223" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B26" s="249">
+        <v>23</v>
+      </c>
+      <c r="C26" s="250" t="s">
+        <v>863</v>
+      </c>
+      <c r="D26" s="251" t="s">
+        <v>864</v>
+      </c>
+      <c r="E26" s="251" t="s">
+        <v>865</v>
+      </c>
+      <c r="F26" s="251" t="s">
+        <v>866</v>
+      </c>
+      <c r="G26" s="252" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="253">
+        <v>24</v>
+      </c>
+      <c r="C27" s="254" t="s">
+        <v>868</v>
+      </c>
+      <c r="D27" s="255" t="s">
+        <v>869</v>
+      </c>
+      <c r="E27" s="255" t="s">
+        <v>870</v>
+      </c>
+      <c r="F27" s="255" t="s">
+        <v>871</v>
+      </c>
+      <c r="G27" s="256" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="253">
+        <v>25</v>
+      </c>
+      <c r="C28" s="254" t="s">
+        <v>873</v>
+      </c>
+      <c r="D28" s="255" t="s">
+        <v>874</v>
+      </c>
+      <c r="E28" s="255" t="s">
+        <v>875</v>
+      </c>
+      <c r="F28" s="255" t="s">
+        <v>876</v>
+      </c>
+      <c r="G28" s="256" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="239">
+        <v>26</v>
+      </c>
+      <c r="C29" s="240" t="s">
+        <v>878</v>
+      </c>
+      <c r="D29" s="241" t="s">
+        <v>879</v>
+      </c>
+      <c r="E29" s="241" t="s">
+        <v>880</v>
+      </c>
+      <c r="F29" s="241" t="s">
+        <v>881</v>
+      </c>
+      <c r="G29" s="242" t="s">
+        <v>882</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="239">
+        <v>27</v>
+      </c>
+      <c r="C30" s="240" t="s">
+        <v>883</v>
+      </c>
+      <c r="D30" s="241" t="s">
+        <v>884</v>
+      </c>
+      <c r="E30" s="241" t="s">
+        <v>885</v>
+      </c>
+      <c r="F30" s="241" t="s">
+        <v>886</v>
+      </c>
+      <c r="G30" s="242" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="239">
+        <v>28</v>
+      </c>
+      <c r="C31" s="240" t="s">
+        <v>888</v>
+      </c>
+      <c r="D31" s="241" t="s">
+        <v>889</v>
+      </c>
+      <c r="E31" s="241" t="s">
+        <v>890</v>
+      </c>
+      <c r="F31" s="241" t="s">
+        <v>891</v>
+      </c>
+      <c r="G31" s="242" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="243">
+        <v>29</v>
+      </c>
+      <c r="C32" s="244" t="s">
+        <v>893</v>
+      </c>
+      <c r="D32" s="241" t="s">
+        <v>894</v>
+      </c>
+      <c r="E32" s="241" t="s">
+        <v>895</v>
+      </c>
+      <c r="F32" s="241" t="s">
+        <v>896</v>
+      </c>
+      <c r="G32" s="242" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B33" s="234" t="s">
+        <v>898</v>
+      </c>
+      <c r="C33" s="235"/>
+      <c r="D33" s="235"/>
+      <c r="E33" s="235"/>
+      <c r="F33" s="235"/>
+      <c r="G33" s="236"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B33:G33"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98DC9442-C99E-46AE-BA24-6CDCF6B108E6}">
+  <dimension ref="A1:N54"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="6" max="6" width="11.5703125" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" customWidth="1"/>
+    <col min="11" max="11" width="13.140625" customWidth="1"/>
+    <col min="12" max="12" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="237" t="s">
+        <v>899</v>
+      </c>
+      <c r="C3" s="237"/>
+      <c r="D3" s="237"/>
+      <c r="F3" s="210" t="s">
+        <v>828</v>
+      </c>
+      <c r="G3" s="210"/>
+      <c r="H3" s="210"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B4" s="238">
+        <f t="shared" ref="B4:D13" ca="1" si="0">RAND()</f>
+        <v>0.32698667282947025</v>
+      </c>
+      <c r="C4" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.39208112969267306</v>
+      </c>
+      <c r="D4" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.99664361027787773</v>
+      </c>
+      <c r="F4" s="167" t="s">
+        <v>901</v>
+      </c>
+      <c r="G4" s="167" t="s">
+        <v>902</v>
+      </c>
+      <c r="H4" s="167" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="238">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.8818701781638848</v>
+      </c>
+      <c r="C5" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.75295636141959676</v>
+      </c>
+      <c r="D5" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.81008471164245044</v>
+      </c>
+      <c r="F5" s="169">
+        <v>1</v>
+      </c>
+      <c r="G5" s="168">
+        <v>186.74647918864025</v>
+      </c>
+      <c r="H5" s="168">
+        <f>ROUND(G5,3)</f>
+        <v>186.74600000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="238">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.31843013867584613</v>
+      </c>
+      <c r="C6" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.63099075127251358</v>
+      </c>
+      <c r="D6" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.17966725671296624</v>
+      </c>
+      <c r="F6" s="169">
+        <v>2</v>
+      </c>
+      <c r="G6" s="168">
+        <v>1134.2033634091172</v>
+      </c>
+      <c r="H6" s="168">
+        <f t="shared" ref="H6:H14" si="1">ROUND(G6,3)</f>
+        <v>1134.203</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="238">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.92087537902698624</v>
+      </c>
+      <c r="C7" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.56418456243774495</v>
+      </c>
+      <c r="D7" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.66945485273370331</v>
+      </c>
+      <c r="F7" s="169">
+        <v>3</v>
+      </c>
+      <c r="G7" s="168">
+        <v>1056.2609033230992</v>
+      </c>
+      <c r="H7" s="168">
+        <f t="shared" si="1"/>
+        <v>1056.261</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="238">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.65034241806481452</v>
+      </c>
+      <c r="C8" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.65197524793134842</v>
+      </c>
+      <c r="D8" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.15855812372165234</v>
+      </c>
+      <c r="F8" s="169">
+        <v>4</v>
+      </c>
+      <c r="G8" s="168">
+        <v>444.95536951220424</v>
+      </c>
+      <c r="H8" s="168">
+        <f t="shared" si="1"/>
+        <v>444.95499999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="238">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.31658206223851315</v>
+      </c>
+      <c r="C9" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.96660832114640227</v>
+      </c>
+      <c r="D9" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.17204586106086683</v>
+      </c>
+      <c r="F9" s="169">
+        <v>5</v>
+      </c>
+      <c r="G9" s="168">
+        <v>1319.4698803550457</v>
+      </c>
+      <c r="H9" s="168">
+        <f t="shared" si="1"/>
+        <v>1319.47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="238">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.33164581465508591</v>
+      </c>
+      <c r="C10" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.71822268545399026</v>
+      </c>
+      <c r="D10" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.358132243878444</v>
+      </c>
+      <c r="F10" s="169">
+        <v>6</v>
+      </c>
+      <c r="G10" s="168">
+        <v>226.9273016860318</v>
+      </c>
+      <c r="H10" s="168">
+        <f t="shared" si="1"/>
+        <v>226.92699999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="238">
+        <f t="shared" ca="1" si="0"/>
+        <v>5.6275228454598425E-2</v>
+      </c>
+      <c r="C11" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.55696991991165046</v>
+      </c>
+      <c r="D11" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.57504254004784972</v>
+      </c>
+      <c r="F11" s="169">
+        <v>7</v>
+      </c>
+      <c r="G11" s="168">
+        <v>130.1594492248114</v>
+      </c>
+      <c r="H11" s="168">
+        <f t="shared" si="1"/>
+        <v>130.15899999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="238">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.52189944424699652</v>
+      </c>
+      <c r="C12" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.62260756937680262</v>
+      </c>
+      <c r="D12" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.19412747264811814</v>
+      </c>
+      <c r="F12" s="169">
+        <v>8</v>
+      </c>
+      <c r="G12" s="168">
+        <v>351.12731634061288</v>
+      </c>
+      <c r="H12" s="168">
+        <f t="shared" si="1"/>
+        <v>351.12700000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="238">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.5385280325448456</v>
+      </c>
+      <c r="C13" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.30399083487210932</v>
+      </c>
+      <c r="D13" s="168">
+        <f t="shared" ca="1" si="0"/>
+        <v>0.70723732570769393</v>
+      </c>
+      <c r="F13" s="169">
+        <v>9</v>
+      </c>
+      <c r="G13" s="168">
+        <v>1433.0594361477456</v>
+      </c>
+      <c r="H13" s="168">
+        <f t="shared" si="1"/>
+        <v>1433.059</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="F14" s="169">
+        <v>10</v>
+      </c>
+      <c r="G14" s="168">
+        <v>214.62573845192333</v>
+      </c>
+      <c r="H14" s="168">
+        <f t="shared" si="1"/>
+        <v>214.626</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B17" s="237" t="s">
+        <v>900</v>
+      </c>
+      <c r="C17" s="237"/>
+      <c r="D17" s="237"/>
+      <c r="F17" s="210" t="s">
+        <v>903</v>
+      </c>
+      <c r="G17" s="210"/>
+      <c r="H17" s="210"/>
+      <c r="J17" s="210" t="s">
+        <v>906</v>
+      </c>
+      <c r="K17" s="210"/>
+      <c r="L17" s="210"/>
+      <c r="M17" s="210"/>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B18" s="238">
+        <f ca="1">RANDBETWEEN(0,100)</f>
+        <v>42</v>
+      </c>
+      <c r="C18" s="168">
+        <f t="shared" ref="B18:D27" ca="1" si="2">RANDBETWEEN(0,100)</f>
+        <v>43</v>
+      </c>
+      <c r="D18" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>31</v>
+      </c>
+      <c r="F18" s="167" t="s">
+        <v>901</v>
+      </c>
+      <c r="G18" s="167" t="s">
+        <v>902</v>
+      </c>
+      <c r="H18" s="167" t="s">
+        <v>903</v>
+      </c>
+      <c r="J18" s="167" t="s">
+        <v>901</v>
+      </c>
+      <c r="K18" s="167" t="s">
+        <v>902</v>
+      </c>
+      <c r="L18" s="167" t="s">
+        <v>905</v>
+      </c>
+      <c r="M18" s="167" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B19" s="238">
+        <f t="shared" ca="1" si="2"/>
+        <v>98</v>
+      </c>
+      <c r="C19" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>99</v>
+      </c>
+      <c r="D19" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="F19" s="169">
+        <v>1</v>
+      </c>
+      <c r="G19" s="168">
+        <v>186.74647918864025</v>
+      </c>
+      <c r="H19" s="168">
+        <f>ROUNDUP(G19,3)</f>
+        <v>186.74700000000001</v>
+      </c>
+      <c r="J19" s="169">
+        <v>1</v>
+      </c>
+      <c r="K19" s="168">
+        <v>186.74647918864025</v>
+      </c>
+      <c r="L19" s="168">
+        <f>INT(K19)</f>
+        <v>186</v>
+      </c>
+      <c r="M19" s="168">
+        <f>TRUNC(K19,1)</f>
+        <v>186.7</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B20" s="238">
+        <f t="shared" ca="1" si="2"/>
+        <v>56</v>
+      </c>
+      <c r="C20" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="D20" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>46</v>
+      </c>
+      <c r="F20" s="169">
+        <v>2</v>
+      </c>
+      <c r="G20" s="168">
+        <v>1134.2033634091172</v>
+      </c>
+      <c r="H20" s="168">
+        <f t="shared" ref="H20:H28" si="3">ROUNDUP(G20,3)</f>
+        <v>1134.204</v>
+      </c>
+      <c r="J20" s="169">
+        <v>2</v>
+      </c>
+      <c r="K20" s="168">
+        <v>1134.2033634091172</v>
+      </c>
+      <c r="L20" s="168">
+        <f t="shared" ref="L20:L28" si="4">INT(K20)</f>
+        <v>1134</v>
+      </c>
+      <c r="M20" s="168">
+        <f t="shared" ref="M20:M28" si="5">TRUNC(K20,1)</f>
+        <v>1134.2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B21" s="238">
+        <f t="shared" ca="1" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="C21" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>56</v>
+      </c>
+      <c r="D21" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>59</v>
+      </c>
+      <c r="F21" s="169">
+        <v>3</v>
+      </c>
+      <c r="G21" s="168">
+        <v>1056.2609033230992</v>
+      </c>
+      <c r="H21" s="168">
+        <f t="shared" si="3"/>
+        <v>1056.261</v>
+      </c>
+      <c r="J21" s="169">
+        <v>3</v>
+      </c>
+      <c r="K21" s="168">
+        <v>1056.2609033230992</v>
+      </c>
+      <c r="L21" s="168">
+        <f t="shared" si="4"/>
+        <v>1056</v>
+      </c>
+      <c r="M21" s="168">
+        <f t="shared" si="5"/>
+        <v>1056.2</v>
+      </c>
+    </row>
+    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B22" s="238">
+        <f t="shared" ca="1" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="C22" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="D22" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="F22" s="169">
+        <v>4</v>
+      </c>
+      <c r="G22" s="168">
+        <v>444.95536951220424</v>
+      </c>
+      <c r="H22" s="168">
+        <f t="shared" si="3"/>
+        <v>444.95599999999996</v>
+      </c>
+      <c r="J22" s="169">
+        <v>4</v>
+      </c>
+      <c r="K22" s="168">
+        <v>444.95536951220424</v>
+      </c>
+      <c r="L22" s="168">
+        <f t="shared" si="4"/>
+        <v>444</v>
+      </c>
+      <c r="M22" s="168">
+        <f t="shared" si="5"/>
+        <v>444.9</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B23" s="238">
+        <f t="shared" ca="1" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="C23" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>84</v>
+      </c>
+      <c r="D23" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>27</v>
+      </c>
+      <c r="F23" s="169">
+        <v>5</v>
+      </c>
+      <c r="G23" s="168">
+        <v>1319.4698803550457</v>
+      </c>
+      <c r="H23" s="168">
+        <f t="shared" si="3"/>
+        <v>1319.47</v>
+      </c>
+      <c r="J23" s="169">
+        <v>5</v>
+      </c>
+      <c r="K23" s="168">
+        <v>1319.4698803550457</v>
+      </c>
+      <c r="L23" s="168">
+        <f t="shared" si="4"/>
+        <v>1319</v>
+      </c>
+      <c r="M23" s="168">
+        <f t="shared" si="5"/>
+        <v>1319.4</v>
+      </c>
+    </row>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B24" s="238">
+        <f t="shared" ca="1" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="C24" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="D24" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>89</v>
+      </c>
+      <c r="F24" s="169">
+        <v>6</v>
+      </c>
+      <c r="G24" s="168">
+        <v>226.9273016860318</v>
+      </c>
+      <c r="H24" s="168">
+        <f t="shared" si="3"/>
+        <v>226.928</v>
+      </c>
+      <c r="J24" s="169">
+        <v>6</v>
+      </c>
+      <c r="K24" s="168">
+        <v>226.9273016860318</v>
+      </c>
+      <c r="L24" s="168">
+        <f t="shared" si="4"/>
+        <v>226</v>
+      </c>
+      <c r="M24" s="168">
+        <f t="shared" si="5"/>
+        <v>226.9</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B25" s="238">
+        <f t="shared" ca="1" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="C25" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>44</v>
+      </c>
+      <c r="D25" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>93</v>
+      </c>
+      <c r="F25" s="169">
+        <v>7</v>
+      </c>
+      <c r="G25" s="168">
+        <v>130.1594492248114</v>
+      </c>
+      <c r="H25" s="168">
+        <f t="shared" si="3"/>
+        <v>130.16</v>
+      </c>
+      <c r="J25" s="169">
+        <v>7</v>
+      </c>
+      <c r="K25" s="168">
+        <v>130.1594492248114</v>
+      </c>
+      <c r="L25" s="168">
+        <f t="shared" si="4"/>
+        <v>130</v>
+      </c>
+      <c r="M25" s="168">
+        <f t="shared" si="5"/>
+        <v>130.1</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B26" s="238">
+        <f t="shared" ca="1" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="C26" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>47</v>
+      </c>
+      <c r="D26" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>64</v>
+      </c>
+      <c r="F26" s="169">
+        <v>8</v>
+      </c>
+      <c r="G26" s="168">
+        <v>351.12731634061288</v>
+      </c>
+      <c r="H26" s="168">
+        <f t="shared" si="3"/>
+        <v>351.12799999999999</v>
+      </c>
+      <c r="J26" s="169">
+        <v>8</v>
+      </c>
+      <c r="K26" s="168">
+        <v>351.12731634061288</v>
+      </c>
+      <c r="L26" s="168">
+        <f t="shared" si="4"/>
+        <v>351</v>
+      </c>
+      <c r="M26" s="168">
+        <f t="shared" si="5"/>
+        <v>351.1</v>
+      </c>
+    </row>
+    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B27" s="238">
+        <f t="shared" ca="1" si="2"/>
+        <v>18</v>
+      </c>
+      <c r="C27" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="D27" s="168">
+        <f t="shared" ca="1" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="F27" s="169">
+        <v>9</v>
+      </c>
+      <c r="G27" s="168">
+        <v>1433.0594361477456</v>
+      </c>
+      <c r="H27" s="168">
+        <f t="shared" si="3"/>
+        <v>1433.06</v>
+      </c>
+      <c r="J27" s="169">
+        <v>9</v>
+      </c>
+      <c r="K27" s="168">
+        <v>1433.0594361477456</v>
+      </c>
+      <c r="L27" s="168">
+        <f t="shared" si="4"/>
+        <v>1433</v>
+      </c>
+      <c r="M27" s="168">
+        <f t="shared" si="5"/>
+        <v>1433</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="F28" s="169">
+        <v>10</v>
+      </c>
+      <c r="G28" s="168">
+        <v>214.62573845192333</v>
+      </c>
+      <c r="H28" s="168">
+        <f t="shared" si="3"/>
+        <v>214.626</v>
+      </c>
+      <c r="J28" s="169">
+        <v>10</v>
+      </c>
+      <c r="K28" s="168">
+        <v>214.62573845192333</v>
+      </c>
+      <c r="L28" s="168">
+        <f t="shared" si="4"/>
+        <v>214</v>
+      </c>
+      <c r="M28" s="168">
+        <f t="shared" si="5"/>
+        <v>214.6</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B30" s="237" t="s">
+        <v>873</v>
+      </c>
+      <c r="C30" s="237"/>
+      <c r="D30" s="237"/>
+      <c r="F30" s="210" t="s">
+        <v>904</v>
+      </c>
+      <c r="G30" s="210"/>
+      <c r="H30" s="210"/>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B31" s="238" cm="1">
+        <f t="array" aca="1" ref="B31:D40" ca="1">_xlfn.RANDARRAY(10,3,0,100,TRUE)</f>
+        <v>89</v>
+      </c>
+      <c r="C31" s="168">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
+      <c r="D31" s="168">
+        <f ca="1"/>
+        <v>27</v>
+      </c>
+      <c r="F31" s="167" t="s">
+        <v>901</v>
+      </c>
+      <c r="G31" s="167" t="s">
+        <v>902</v>
+      </c>
+      <c r="H31" s="167" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B32" s="238">
+        <f ca="1"/>
+        <v>34</v>
+      </c>
+      <c r="C32" s="168">
+        <f ca="1"/>
+        <v>75</v>
+      </c>
+      <c r="D32" s="168">
+        <f ca="1"/>
+        <v>78</v>
+      </c>
+      <c r="F32" s="169">
+        <v>1</v>
+      </c>
+      <c r="G32" s="168">
+        <v>186.74647918864025</v>
+      </c>
+      <c r="H32" s="168">
+        <f>ROUNDDOWN(G32,3)</f>
+        <v>186.74600000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B33" s="238">
+        <f ca="1"/>
+        <v>28</v>
+      </c>
+      <c r="C33" s="168">
+        <f ca="1"/>
+        <v>37</v>
+      </c>
+      <c r="D33" s="168">
+        <f ca="1"/>
+        <v>54</v>
+      </c>
+      <c r="F33" s="169">
+        <v>2</v>
+      </c>
+      <c r="G33" s="168">
+        <v>1134.2033634091172</v>
+      </c>
+      <c r="H33" s="168">
+        <f t="shared" ref="H33:H41" si="6">ROUNDDOWN(G33,3)</f>
+        <v>1134.203</v>
+      </c>
+      <c r="N33" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B34" s="238">
+        <f ca="1"/>
+        <v>5</v>
+      </c>
+      <c r="C34" s="168">
+        <f ca="1"/>
+        <v>19</v>
+      </c>
+      <c r="D34" s="168">
+        <f ca="1"/>
+        <v>72</v>
+      </c>
+      <c r="F34" s="169">
+        <v>3</v>
+      </c>
+      <c r="G34" s="168">
+        <v>1056.2609033230992</v>
+      </c>
+      <c r="H34" s="168">
+        <f t="shared" si="6"/>
+        <v>1056.26</v>
+      </c>
+    </row>
+    <row r="35" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B35" s="238">
+        <f ca="1"/>
+        <v>97</v>
+      </c>
+      <c r="C35" s="168">
+        <f ca="1"/>
+        <v>87</v>
+      </c>
+      <c r="D35" s="168">
+        <f ca="1"/>
+        <v>58</v>
+      </c>
+      <c r="F35" s="169">
+        <v>4</v>
+      </c>
+      <c r="G35" s="168">
+        <v>444.95536951220424</v>
+      </c>
+      <c r="H35" s="168">
+        <f t="shared" si="6"/>
+        <v>444.95499999999998</v>
+      </c>
+    </row>
+    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B36" s="238">
+        <f ca="1"/>
+        <v>6</v>
+      </c>
+      <c r="C36" s="168">
+        <f ca="1"/>
+        <v>6</v>
+      </c>
+      <c r="D36" s="168">
+        <f ca="1"/>
+        <v>41</v>
+      </c>
+      <c r="F36" s="169">
+        <v>5</v>
+      </c>
+      <c r="G36" s="168">
+        <v>1319.4698803550457</v>
+      </c>
+      <c r="H36" s="168">
+        <f t="shared" si="6"/>
+        <v>1319.4690000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B37" s="238">
+        <f ca="1"/>
+        <v>88</v>
+      </c>
+      <c r="C37" s="168">
+        <f ca="1"/>
+        <v>74</v>
+      </c>
+      <c r="D37" s="168">
+        <f ca="1"/>
+        <v>60</v>
+      </c>
+      <c r="F37" s="169">
+        <v>6</v>
+      </c>
+      <c r="G37" s="168">
+        <v>226.9273016860318</v>
+      </c>
+      <c r="H37" s="168">
+        <f t="shared" si="6"/>
+        <v>226.92699999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B38" s="238">
+        <f ca="1"/>
+        <v>17</v>
+      </c>
+      <c r="C38" s="168">
+        <f ca="1"/>
+        <v>60</v>
+      </c>
+      <c r="D38" s="168">
+        <f ca="1"/>
+        <v>89</v>
+      </c>
+      <c r="F38" s="169">
+        <v>7</v>
+      </c>
+      <c r="G38" s="168">
+        <v>130.1594492248114</v>
+      </c>
+      <c r="H38" s="168">
+        <f t="shared" si="6"/>
+        <v>130.15899999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B39" s="238">
+        <f ca="1"/>
+        <v>0</v>
+      </c>
+      <c r="C39" s="168">
+        <f ca="1"/>
+        <v>33</v>
+      </c>
+      <c r="D39" s="168">
+        <f ca="1"/>
+        <v>9</v>
+      </c>
+      <c r="F39" s="169">
+        <v>8</v>
+      </c>
+      <c r="G39" s="168">
+        <v>351.12731634061288</v>
+      </c>
+      <c r="H39" s="168">
+        <f t="shared" si="6"/>
+        <v>351.12700000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B40" s="238">
+        <f ca="1"/>
+        <v>81</v>
+      </c>
+      <c r="C40" s="168">
+        <f ca="1"/>
+        <v>7</v>
+      </c>
+      <c r="D40" s="168">
+        <f ca="1"/>
+        <v>71</v>
+      </c>
+      <c r="F40" s="169">
+        <v>9</v>
+      </c>
+      <c r="G40" s="168">
+        <v>1433.0594361477456</v>
+      </c>
+      <c r="H40" s="168">
+        <f t="shared" si="6"/>
+        <v>1433.059</v>
+      </c>
+    </row>
+    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="F41" s="169">
+        <v>10</v>
+      </c>
+      <c r="G41" s="168">
+        <v>214.62573845192333</v>
+      </c>
+      <c r="H41" s="168">
+        <f t="shared" si="6"/>
+        <v>214.625</v>
+      </c>
+    </row>
+    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B43" s="210" t="s">
+        <v>813</v>
+      </c>
+      <c r="C43" s="210"/>
+      <c r="D43" s="210"/>
+      <c r="F43" s="210" t="s">
+        <v>818</v>
+      </c>
+      <c r="G43" s="210"/>
+      <c r="H43" s="210"/>
+    </row>
+    <row r="44" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B44" s="167" t="s">
+        <v>901</v>
+      </c>
+      <c r="C44" s="167" t="s">
+        <v>902</v>
+      </c>
+      <c r="D44" s="167" t="s">
+        <v>813</v>
+      </c>
+      <c r="F44" s="167" t="s">
+        <v>901</v>
+      </c>
+      <c r="G44" s="167" t="s">
+        <v>902</v>
+      </c>
+      <c r="H44" s="167" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="45" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B45" s="169">
+        <v>1</v>
+      </c>
+      <c r="C45" s="168">
+        <v>821</v>
+      </c>
+      <c r="D45" s="168">
+        <v>942</v>
+      </c>
+      <c r="F45" s="169">
+        <v>1</v>
+      </c>
+      <c r="G45" s="238">
+        <v>821</v>
+      </c>
+      <c r="H45" s="168" cm="1">
+        <f t="array" ref="H45:H54">SMALL($G$45:$G$54,F45:F54)</f>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B46" s="169">
+        <v>2</v>
+      </c>
+      <c r="C46" s="168">
+        <v>486</v>
+      </c>
+      <c r="D46" s="168">
+        <v>821</v>
+      </c>
+      <c r="F46" s="169">
+        <v>2</v>
+      </c>
+      <c r="G46" s="238">
+        <v>486</v>
+      </c>
+      <c r="H46" s="168">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B47" s="169">
+        <v>3</v>
+      </c>
+      <c r="C47" s="168">
+        <v>528</v>
+      </c>
+      <c r="D47" s="168">
+        <v>813</v>
+      </c>
+      <c r="F47" s="169">
+        <v>3</v>
+      </c>
+      <c r="G47" s="238">
+        <v>528</v>
+      </c>
+      <c r="H47" s="168">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B48" s="169">
+        <v>4</v>
+      </c>
+      <c r="C48" s="168">
+        <v>128</v>
+      </c>
+      <c r="D48" s="168">
+        <v>528</v>
+      </c>
+      <c r="F48" s="169">
+        <v>4</v>
+      </c>
+      <c r="G48" s="238">
+        <v>128</v>
+      </c>
+      <c r="H48" s="168">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="49" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B49" s="169">
+        <v>5</v>
+      </c>
+      <c r="C49" s="168">
+        <v>422</v>
+      </c>
+      <c r="D49" s="168">
+        <v>486</v>
+      </c>
+      <c r="F49" s="169">
+        <v>5</v>
+      </c>
+      <c r="G49" s="238">
+        <v>422</v>
+      </c>
+      <c r="H49" s="168">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="50" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B50" s="169">
+        <v>6</v>
+      </c>
+      <c r="C50" s="168">
+        <v>206</v>
+      </c>
+      <c r="D50" s="168">
+        <v>422</v>
+      </c>
+      <c r="F50" s="169">
+        <v>6</v>
+      </c>
+      <c r="G50" s="238">
+        <v>206</v>
+      </c>
+      <c r="H50" s="168">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="51" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B51" s="169">
+        <v>7</v>
+      </c>
+      <c r="C51" s="168">
+        <v>942</v>
+      </c>
+      <c r="D51" s="168">
+        <v>330</v>
+      </c>
+      <c r="F51" s="169">
+        <v>7</v>
+      </c>
+      <c r="G51" s="238">
+        <v>942</v>
+      </c>
+      <c r="H51" s="168">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="52" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B52" s="169">
+        <v>8</v>
+      </c>
+      <c r="C52" s="168">
+        <v>296</v>
+      </c>
+      <c r="D52" s="168">
+        <v>296</v>
+      </c>
+      <c r="F52" s="169">
+        <v>8</v>
+      </c>
+      <c r="G52" s="238">
+        <v>296</v>
+      </c>
+      <c r="H52" s="168">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="53" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B53" s="169">
+        <v>9</v>
+      </c>
+      <c r="C53" s="168">
+        <v>813</v>
+      </c>
+      <c r="D53" s="168">
+        <v>206</v>
+      </c>
+      <c r="F53" s="169">
+        <v>9</v>
+      </c>
+      <c r="G53" s="238">
+        <v>813</v>
+      </c>
+      <c r="H53" s="168">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="54" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B54" s="169">
+        <v>10</v>
+      </c>
+      <c r="C54" s="168">
+        <v>330</v>
+      </c>
+      <c r="D54" s="168">
+        <v>128</v>
+      </c>
+      <c r="F54" s="169">
+        <v>10</v>
+      </c>
+      <c r="G54" s="238">
+        <v>330</v>
+      </c>
+      <c r="H54" s="168">
+        <v>942</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="F43:H43"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="J17:M17"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="B43:D43"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C45:C54">
+    <cfRule type="top10" dxfId="8" priority="6" rank="3"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G45:G54">
+    <cfRule type="top10" dxfId="4" priority="2" bottom="1" rank="3"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E70BB3C3-248D-45A3-AA24-450B5755F8CE}">
   <dimension ref="A1:N43"/>
@@ -28532,11 +31383,11 @@
       </c>
       <c r="D2" s="25">
         <f t="shared" ref="C2:F15" ca="1" si="0">RANDBETWEEN(0,100)</f>
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="E2" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <v>70</v>
       </c>
       <c r="F2" s="25"/>
       <c r="G2" s="28">
@@ -28558,16 +31409,16 @@
       </c>
       <c r="C3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="D3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="E3" s="25"/>
       <c r="F3" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="G3" s="28">
         <f t="shared" ref="G3:G15" ca="1" si="1">COUNT(C3:F3)</f>
@@ -28589,11 +31440,11 @@
       <c r="C4" s="25"/>
       <c r="D4" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E4" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="F4" s="25"/>
       <c r="G4" s="28">
@@ -28615,16 +31466,16 @@
       </c>
       <c r="C5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>51</v>
+        <v>67</v>
       </c>
       <c r="E5" s="25"/>
       <c r="F5" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="G5" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28645,16 +31496,16 @@
       </c>
       <c r="C6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="D6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>3</v>
       </c>
       <c r="E6" s="25"/>
       <c r="F6" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>54</v>
+        <v>3</v>
       </c>
       <c r="G6" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28676,15 +31527,15 @@
       <c r="C7" s="25"/>
       <c r="D7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="E7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F7" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="G7" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28705,7 +31556,7 @@
       </c>
       <c r="C8" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>50</v>
       </c>
       <c r="D8" s="25" t="s">
         <v>468</v>
@@ -28715,7 +31566,7 @@
       </c>
       <c r="F8" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="G8" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28736,19 +31587,19 @@
       </c>
       <c r="C9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="D9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="E9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>89</v>
       </c>
       <c r="F9" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="G9" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28774,7 +31625,7 @@
       <c r="D10" s="25"/>
       <c r="E10" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>56</v>
+        <v>91</v>
       </c>
       <c r="F10" s="25"/>
       <c r="G10" s="28">
@@ -28796,19 +31647,19 @@
       </c>
       <c r="C11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>12</v>
       </c>
       <c r="D11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="E11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="F11" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G11" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28829,15 +31680,15 @@
       </c>
       <c r="C12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>64</v>
+        <v>97</v>
       </c>
       <c r="D12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="E12" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="F12" s="25"/>
       <c r="G12" s="28">
@@ -28859,16 +31710,16 @@
       </c>
       <c r="C13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="D13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="E13" s="25"/>
       <c r="F13" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="G13" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28889,18 +31740,18 @@
       </c>
       <c r="C14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="D14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="E14" s="25" t="s">
         <v>468</v>
       </c>
       <c r="F14" s="25">
         <f t="shared" ca="1" si="0"/>
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G14" s="28">
         <f t="shared" ca="1" si="1"/>
@@ -28925,7 +31776,7 @@
       <c r="D15" s="27"/>
       <c r="E15" s="27">
         <f t="shared" ca="1" si="0"/>
-        <v>67</v>
+        <v>94</v>
       </c>
       <c r="F15" s="27" t="s">
         <v>468</v>
@@ -33362,54 +36213,54 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E51">
-    <cfRule type="cellIs" dxfId="57" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="72" priority="44" operator="equal">
       <formula>20000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="45" operator="between">
+    <cfRule type="cellIs" dxfId="71" priority="45" operator="between">
       <formula>50000</formula>
       <formula>100000</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="55" priority="46" operator="between">
+    <cfRule type="cellIs" dxfId="70" priority="46" operator="between">
       <formula>"Rs. 65,984"</formula>
       <formula>"Rs. 121,395"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="47" operator="lessThan">
+    <cfRule type="cellIs" dxfId="69" priority="47" operator="lessThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="53" priority="48" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="68" priority="48" operator="greaterThan">
       <formula>93689</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="49" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="67" priority="49" operator="greaterThan">
       <formula>"Rs. 93,689"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B53">
-    <cfRule type="containsText" dxfId="51" priority="43" operator="containsText" text="Ayesha khan">
+    <cfRule type="containsText" dxfId="66" priority="43" operator="containsText" text="Ayesha khan">
       <formula>NOT(ISERROR(SEARCH("Ayesha khan",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A3:A53">
-    <cfRule type="timePeriod" dxfId="50" priority="41" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="65" priority="41" timePeriod="yesterday">
       <formula>FLOOR(A3,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="49" priority="42" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="64" priority="42" timePeriod="yesterday">
       <formula>FLOOR(A3,1)=TODAY()-1</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:A53">
-    <cfRule type="timePeriod" dxfId="48" priority="38" timePeriod="nextWeek">
+    <cfRule type="timePeriod" dxfId="63" priority="38" timePeriod="nextWeek">
       <formula>AND(ROUNDDOWN(A2,0)-TODAY()&gt;(7-WEEKDAY(TODAY())),ROUNDDOWN(A2,0)-TODAY()&lt;(15-WEEKDAY(TODAY())))</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="47" priority="39" timePeriod="yesterday">
+    <cfRule type="timePeriod" dxfId="62" priority="39" timePeriod="yesterday">
       <formula>FLOOR(A2,1)=TODAY()-1</formula>
     </cfRule>
-    <cfRule type="timePeriod" dxfId="46" priority="40" timePeriod="today">
+    <cfRule type="timePeriod" dxfId="61" priority="40" timePeriod="today">
       <formula>FLOOR(A2,1)=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F53">
-    <cfRule type="uniqueValues" dxfId="45" priority="36"/>
-    <cfRule type="duplicateValues" dxfId="44" priority="37"/>
+    <cfRule type="uniqueValues" dxfId="60" priority="36"/>
+    <cfRule type="duplicateValues" dxfId="59" priority="37"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E55:E105">
     <cfRule type="dataBar" priority="18">

</xml_diff>